<commit_message>
replace bank flows with synthetic case data
</commit_message>
<xml_diff>
--- a/data/processed/name_mapping.xlsx
+++ b/data/processed/name_mapping.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,36 +431,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>周芷</t>
+          <t>张三</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>杨周武之妻何晓初</t>
+          <t>王静</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>张三</t>
+          <t>李四</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>王静</t>
+          <t>杨周武</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>张夏天</t>
+          <t>老刘</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>王静</t>
+          <t>刘力飚</t>
         </is>
       </c>
     </row>
@@ -472,55 +472,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>杨周武之妻何晓初</t>
+          <t>何晓初</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>李四</t>
+          <t>饶蝶</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>杨周武</t>
+          <t>何晓初控制账户</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>罗宇</t>
+          <t>周芷</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>王静</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>陈三一</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>王静</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>饶蝶</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>杨周武之妻何晓初</t>
+          <t>何晓初控制账户</t>
         </is>
       </c>
     </row>

</xml_diff>